<commit_message>
Add backfill scripts for BLF returns and historical data collection
- Created `back_fill_history.py` for backfilling BLF returns data from PDFs.
- Implemented functions for downloading PDFs, parsing data, and saving to Excel.
- Added `backfill_all_history.py` for comprehensive historical data collection.
- Introduced data validation and cleaning functions to ensure data integrity.
- Generated temporary Excel file for backfilled data.
</commit_message>
<xml_diff>
--- a/blf_returns.xlsx
+++ b/blf_returns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\爬蟲專案\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B2DA21-F7F0-4934-9774-56E8FC1D69DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D37DE4A7-E584-4C53-9254-A927462CECCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4308" yWindow="1500" windowWidth="17280" windowHeight="9984" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
   <si>
     <t>年月</t>
   </si>
@@ -362,6 +362,9 @@
   </si>
   <si>
     <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
   </si>
 </sst>
 </file>
@@ -733,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr defaultRowHeight="15.3" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -883,6 +886,12 @@
       <c r="E8">
         <v>0</v>
       </c>
+      <c r="F8">
+        <v>3.82</v>
+      </c>
+      <c r="G8">
+        <v>7.15</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
@@ -1081,6 +1090,12 @@
       <c r="E20">
         <v>0</v>
       </c>
+      <c r="F20">
+        <v>3.16</v>
+      </c>
+      <c r="G20">
+        <v>-1.1399999999999999</v>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
@@ -1279,6 +1294,12 @@
       <c r="E32">
         <v>0</v>
       </c>
+      <c r="F32">
+        <v>3.6</v>
+      </c>
+      <c r="G32">
+        <v>10.62</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
@@ -1477,6 +1498,12 @@
       <c r="E44">
         <v>0</v>
       </c>
+      <c r="F44">
+        <v>2.31</v>
+      </c>
+      <c r="G44">
+        <v>8.4600000000000009</v>
+      </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
@@ -1807,6 +1834,12 @@
       <c r="E56">
         <v>11.22</v>
       </c>
+      <c r="F56">
+        <v>8.41</v>
+      </c>
+      <c r="G56">
+        <v>11.85</v>
+      </c>
       <c r="H56">
         <v>0.44</v>
       </c>
@@ -2221,6 +2254,12 @@
       <c r="E68">
         <v>-8.3000000000000007</v>
       </c>
+      <c r="F68">
+        <v>1.95</v>
+      </c>
+      <c r="G68">
+        <v>-6.73</v>
+      </c>
       <c r="H68">
         <v>1.23</v>
       </c>
@@ -2635,6 +2674,12 @@
       <c r="E80">
         <v>14.83</v>
       </c>
+      <c r="F80">
+        <v>3.47</v>
+      </c>
+      <c r="G80">
+        <v>13.1</v>
+      </c>
       <c r="H80">
         <v>1.21</v>
       </c>
@@ -3049,6 +3094,12 @@
       <c r="E92">
         <v>19.36</v>
       </c>
+      <c r="F92">
+        <v>5.72</v>
+      </c>
+      <c r="G92">
+        <v>17.489999999999998</v>
+      </c>
       <c r="H92">
         <v>1.51</v>
       </c>
@@ -3463,6 +3514,12 @@
       <c r="E104">
         <v>22.53</v>
       </c>
+      <c r="F104">
+        <v>5.57</v>
+      </c>
+      <c r="G104">
+        <v>15.96</v>
+      </c>
       <c r="H104">
         <v>1.47</v>
       </c>
@@ -3474,6 +3531,41 @@
       </c>
       <c r="K104">
         <v>8.17</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="A105" t="s">
+        <v>114</v>
+      </c>
+      <c r="B105">
+        <v>5.16</v>
+      </c>
+      <c r="C105">
+        <v>5.1100000000000003</v>
+      </c>
+      <c r="D105">
+        <v>5.03</v>
+      </c>
+      <c r="E105">
+        <v>8.08</v>
+      </c>
+      <c r="F105">
+        <v>0.74</v>
+      </c>
+      <c r="G105">
+        <v>5.1100000000000003</v>
+      </c>
+      <c r="H105">
+        <v>1.41</v>
+      </c>
+      <c r="I105">
+        <v>10.7</v>
+      </c>
+      <c r="J105">
+        <v>2.96</v>
+      </c>
+      <c r="K105">
+        <v>0.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>